<commit_message>
Dashboard quản trị tài chính & KPI
- 8 tab: tổng quan, doanh thu & margin, khách hàng, dòng tiền, công nợ
  phải thu/phải trả, KPI & hoa hồng, cảnh báo; dựng theo Xperise Design System
- Đơn vị tiền chọn được cho cả trang (VND gốc / nghìn / triệu / tỷ) và số lẻ
- Bấm vào biểu đồ ra danh sách khách đứng sau con số đó
- Sửa công nợ theo khách và theo kỳ trên web, overlay riêng nên upload
  file template không ghi đè; ngày gửi bảng kê nối từ app Reconciliation
- Nhập số tổng thẳng trên dashboard: kế hoạch, GMV & giá vốn, chi phí, dòng tiền
- Cảnh báo kèm số trước → sau: khách giảm doanh thu và margin, khách thu
  tiền chậm lại, khoản chi phí tăng
- Tuổi nợ tính theo ngày hôm nay thay vì ngày chốt số liệu trong file

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UN2dxwdZdvi4fAHHKDZwka
</commit_message>
<xml_diff>
--- a/public/dashboard/templates/Xperise_Dashboard_Template.xlsx
+++ b/public/dashboard/templates/Xperise_Dashboard_Template.xlsx
@@ -23,13 +23,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'THAM_SO'!$A$3:$C$37</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DM_KHACH_HANG'!$A$3:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'DM_KHACH_HANG'!$A$3:$I$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'DM_NCC'!$A$3:$E$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'DM_NHAN_SU'!$A$3:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PHAN_BO_PM'!$A$3:$C$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'KE_HOACH'!$A$3:$P$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'GMV'!$A$3:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CONG_NO_PHAI_THU'!$A$3:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CONG_NO_PHAI_THU'!$A$3:$J$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CONG_NO_PHAI_TRA'!$A$3:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'DONG_TIEN'!$A$3:$D$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'CHI_PHI'!$A$3:$C$4</definedName>
@@ -2902,7 +2902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2912,7 +2912,7 @@
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2967,6 +2967,11 @@
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
+          <t>Mã nhóm đối soát</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
           <t>Ghi chú</t>
         </is>
       </c>
@@ -3140,7 +3145,7 @@
       <c r="G59" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H4"/>
+  <autoFilter ref="A3:I59"/>
   <dataValidations count="1">
     <dataValidation sqref="D4:D20000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Giá trị không hợp lệ" error="Chọn một giá trị trong danh sách" type="list">
       <formula1>"N1,N2,N3,N4,N5"</formula1>
@@ -5996,17 +6001,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:J59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6041,424 +6047,434 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
+          <t>Ngày gửi bảng kê</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
           <t>Ngày hóa đơn</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>Ngày đến hạn *</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Số tiền phải thu *</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>Đã thu</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t>Ngày thu đủ</t>
         </is>
       </c>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>Ngày thu gần nhất</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="D4" s="19" t="n"/>
       <c r="E4" s="19" t="n"/>
-      <c r="F4" s="18" t="n"/>
+      <c r="F4" s="19" t="n"/>
       <c r="G4" s="18" t="n"/>
-      <c r="H4" s="19" t="n"/>
+      <c r="H4" s="18" t="n"/>
+      <c r="I4" s="19" t="n"/>
     </row>
     <row r="5">
-      <c r="D5" s="19" t="n"/>
       <c r="E5" s="19" t="n"/>
-      <c r="F5" s="18" t="n"/>
+      <c r="F5" s="19" t="n"/>
       <c r="G5" s="18" t="n"/>
-      <c r="H5" s="19" t="n"/>
+      <c r="H5" s="18" t="n"/>
+      <c r="I5" s="19" t="n"/>
     </row>
     <row r="6">
-      <c r="D6" s="19" t="n"/>
       <c r="E6" s="19" t="n"/>
-      <c r="F6" s="18" t="n"/>
+      <c r="F6" s="19" t="n"/>
       <c r="G6" s="18" t="n"/>
-      <c r="H6" s="19" t="n"/>
+      <c r="H6" s="18" t="n"/>
+      <c r="I6" s="19" t="n"/>
     </row>
     <row r="7">
-      <c r="D7" s="19" t="n"/>
       <c r="E7" s="19" t="n"/>
-      <c r="F7" s="18" t="n"/>
+      <c r="F7" s="19" t="n"/>
       <c r="G7" s="18" t="n"/>
-      <c r="H7" s="19" t="n"/>
+      <c r="H7" s="18" t="n"/>
+      <c r="I7" s="19" t="n"/>
     </row>
     <row r="8">
-      <c r="D8" s="19" t="n"/>
       <c r="E8" s="19" t="n"/>
-      <c r="F8" s="18" t="n"/>
+      <c r="F8" s="19" t="n"/>
       <c r="G8" s="18" t="n"/>
-      <c r="H8" s="19" t="n"/>
+      <c r="H8" s="18" t="n"/>
+      <c r="I8" s="19" t="n"/>
     </row>
     <row r="9">
-      <c r="D9" s="19" t="n"/>
       <c r="E9" s="19" t="n"/>
-      <c r="F9" s="18" t="n"/>
+      <c r="F9" s="19" t="n"/>
       <c r="G9" s="18" t="n"/>
-      <c r="H9" s="19" t="n"/>
+      <c r="H9" s="18" t="n"/>
+      <c r="I9" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="D10" s="19" t="n"/>
       <c r="E10" s="19" t="n"/>
-      <c r="F10" s="18" t="n"/>
+      <c r="F10" s="19" t="n"/>
       <c r="G10" s="18" t="n"/>
-      <c r="H10" s="19" t="n"/>
+      <c r="H10" s="18" t="n"/>
+      <c r="I10" s="19" t="n"/>
     </row>
     <row r="11">
-      <c r="D11" s="19" t="n"/>
       <c r="E11" s="19" t="n"/>
-      <c r="F11" s="18" t="n"/>
+      <c r="F11" s="19" t="n"/>
       <c r="G11" s="18" t="n"/>
-      <c r="H11" s="19" t="n"/>
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="D12" s="19" t="n"/>
       <c r="E12" s="19" t="n"/>
-      <c r="F12" s="18" t="n"/>
+      <c r="F12" s="19" t="n"/>
       <c r="G12" s="18" t="n"/>
-      <c r="H12" s="19" t="n"/>
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="19" t="n"/>
     </row>
     <row r="13">
-      <c r="D13" s="19" t="n"/>
       <c r="E13" s="19" t="n"/>
-      <c r="F13" s="18" t="n"/>
+      <c r="F13" s="19" t="n"/>
       <c r="G13" s="18" t="n"/>
-      <c r="H13" s="19" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="19" t="n"/>
     </row>
     <row r="14">
-      <c r="D14" s="19" t="n"/>
       <c r="E14" s="19" t="n"/>
-      <c r="F14" s="18" t="n"/>
+      <c r="F14" s="19" t="n"/>
       <c r="G14" s="18" t="n"/>
-      <c r="H14" s="19" t="n"/>
+      <c r="H14" s="18" t="n"/>
+      <c r="I14" s="19" t="n"/>
     </row>
     <row r="15">
-      <c r="D15" s="19" t="n"/>
       <c r="E15" s="19" t="n"/>
-      <c r="F15" s="18" t="n"/>
+      <c r="F15" s="19" t="n"/>
       <c r="G15" s="18" t="n"/>
-      <c r="H15" s="19" t="n"/>
+      <c r="H15" s="18" t="n"/>
+      <c r="I15" s="19" t="n"/>
     </row>
     <row r="16">
-      <c r="D16" s="19" t="n"/>
       <c r="E16" s="19" t="n"/>
-      <c r="F16" s="18" t="n"/>
+      <c r="F16" s="19" t="n"/>
       <c r="G16" s="18" t="n"/>
-      <c r="H16" s="19" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="19" t="n"/>
     </row>
     <row r="17">
-      <c r="D17" s="19" t="n"/>
       <c r="E17" s="19" t="n"/>
-      <c r="F17" s="18" t="n"/>
+      <c r="F17" s="19" t="n"/>
       <c r="G17" s="18" t="n"/>
-      <c r="H17" s="19" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="19" t="n"/>
     </row>
     <row r="18">
-      <c r="D18" s="19" t="n"/>
       <c r="E18" s="19" t="n"/>
-      <c r="F18" s="18" t="n"/>
+      <c r="F18" s="19" t="n"/>
       <c r="G18" s="18" t="n"/>
-      <c r="H18" s="19" t="n"/>
+      <c r="H18" s="18" t="n"/>
+      <c r="I18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="D19" s="19" t="n"/>
       <c r="E19" s="19" t="n"/>
-      <c r="F19" s="18" t="n"/>
+      <c r="F19" s="19" t="n"/>
       <c r="G19" s="18" t="n"/>
-      <c r="H19" s="19" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="19" t="n"/>
     </row>
     <row r="20">
-      <c r="D20" s="19" t="n"/>
       <c r="E20" s="19" t="n"/>
-      <c r="F20" s="18" t="n"/>
+      <c r="F20" s="19" t="n"/>
       <c r="G20" s="18" t="n"/>
-      <c r="H20" s="19" t="n"/>
+      <c r="H20" s="18" t="n"/>
+      <c r="I20" s="19" t="n"/>
     </row>
     <row r="21">
-      <c r="D21" s="19" t="n"/>
       <c r="E21" s="19" t="n"/>
-      <c r="F21" s="18" t="n"/>
+      <c r="F21" s="19" t="n"/>
       <c r="G21" s="18" t="n"/>
-      <c r="H21" s="19" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="19" t="n"/>
     </row>
     <row r="22">
-      <c r="D22" s="19" t="n"/>
       <c r="E22" s="19" t="n"/>
-      <c r="F22" s="18" t="n"/>
+      <c r="F22" s="19" t="n"/>
       <c r="G22" s="18" t="n"/>
-      <c r="H22" s="19" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="19" t="n"/>
     </row>
     <row r="23">
-      <c r="D23" s="19" t="n"/>
       <c r="E23" s="19" t="n"/>
-      <c r="F23" s="18" t="n"/>
+      <c r="F23" s="19" t="n"/>
       <c r="G23" s="18" t="n"/>
-      <c r="H23" s="19" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="19" t="n"/>
     </row>
     <row r="24">
-      <c r="D24" s="19" t="n"/>
       <c r="E24" s="19" t="n"/>
-      <c r="F24" s="18" t="n"/>
+      <c r="F24" s="19" t="n"/>
       <c r="G24" s="18" t="n"/>
-      <c r="H24" s="19" t="n"/>
+      <c r="H24" s="18" t="n"/>
+      <c r="I24" s="19" t="n"/>
     </row>
     <row r="25">
-      <c r="D25" s="19" t="n"/>
       <c r="E25" s="19" t="n"/>
-      <c r="F25" s="18" t="n"/>
+      <c r="F25" s="19" t="n"/>
       <c r="G25" s="18" t="n"/>
-      <c r="H25" s="19" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="19" t="n"/>
     </row>
     <row r="26">
-      <c r="D26" s="19" t="n"/>
       <c r="E26" s="19" t="n"/>
-      <c r="F26" s="18" t="n"/>
+      <c r="F26" s="19" t="n"/>
       <c r="G26" s="18" t="n"/>
-      <c r="H26" s="19" t="n"/>
+      <c r="H26" s="18" t="n"/>
+      <c r="I26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="D27" s="19" t="n"/>
       <c r="E27" s="19" t="n"/>
-      <c r="F27" s="18" t="n"/>
+      <c r="F27" s="19" t="n"/>
       <c r="G27" s="18" t="n"/>
-      <c r="H27" s="19" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="19" t="n"/>
     </row>
     <row r="28">
-      <c r="D28" s="19" t="n"/>
       <c r="E28" s="19" t="n"/>
-      <c r="F28" s="18" t="n"/>
+      <c r="F28" s="19" t="n"/>
       <c r="G28" s="18" t="n"/>
-      <c r="H28" s="19" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="19" t="n"/>
     </row>
     <row r="29">
-      <c r="D29" s="19" t="n"/>
       <c r="E29" s="19" t="n"/>
-      <c r="F29" s="18" t="n"/>
+      <c r="F29" s="19" t="n"/>
       <c r="G29" s="18" t="n"/>
-      <c r="H29" s="19" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="19" t="n"/>
     </row>
     <row r="30">
-      <c r="D30" s="19" t="n"/>
       <c r="E30" s="19" t="n"/>
-      <c r="F30" s="18" t="n"/>
+      <c r="F30" s="19" t="n"/>
       <c r="G30" s="18" t="n"/>
-      <c r="H30" s="19" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="19" t="n"/>
     </row>
     <row r="31">
-      <c r="D31" s="19" t="n"/>
       <c r="E31" s="19" t="n"/>
-      <c r="F31" s="18" t="n"/>
+      <c r="F31" s="19" t="n"/>
       <c r="G31" s="18" t="n"/>
-      <c r="H31" s="19" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="19" t="n"/>
     </row>
     <row r="32">
-      <c r="D32" s="19" t="n"/>
       <c r="E32" s="19" t="n"/>
-      <c r="F32" s="18" t="n"/>
+      <c r="F32" s="19" t="n"/>
       <c r="G32" s="18" t="n"/>
-      <c r="H32" s="19" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="19" t="n"/>
     </row>
     <row r="33">
-      <c r="D33" s="19" t="n"/>
       <c r="E33" s="19" t="n"/>
-      <c r="F33" s="18" t="n"/>
+      <c r="F33" s="19" t="n"/>
       <c r="G33" s="18" t="n"/>
-      <c r="H33" s="19" t="n"/>
+      <c r="H33" s="18" t="n"/>
+      <c r="I33" s="19" t="n"/>
     </row>
     <row r="34">
-      <c r="D34" s="19" t="n"/>
       <c r="E34" s="19" t="n"/>
-      <c r="F34" s="18" t="n"/>
+      <c r="F34" s="19" t="n"/>
       <c r="G34" s="18" t="n"/>
-      <c r="H34" s="19" t="n"/>
+      <c r="H34" s="18" t="n"/>
+      <c r="I34" s="19" t="n"/>
     </row>
     <row r="35">
-      <c r="D35" s="19" t="n"/>
       <c r="E35" s="19" t="n"/>
-      <c r="F35" s="18" t="n"/>
+      <c r="F35" s="19" t="n"/>
       <c r="G35" s="18" t="n"/>
-      <c r="H35" s="19" t="n"/>
+      <c r="H35" s="18" t="n"/>
+      <c r="I35" s="19" t="n"/>
     </row>
     <row r="36">
-      <c r="D36" s="19" t="n"/>
       <c r="E36" s="19" t="n"/>
-      <c r="F36" s="18" t="n"/>
+      <c r="F36" s="19" t="n"/>
       <c r="G36" s="18" t="n"/>
-      <c r="H36" s="19" t="n"/>
+      <c r="H36" s="18" t="n"/>
+      <c r="I36" s="19" t="n"/>
     </row>
     <row r="37">
-      <c r="D37" s="19" t="n"/>
       <c r="E37" s="19" t="n"/>
-      <c r="F37" s="18" t="n"/>
+      <c r="F37" s="19" t="n"/>
       <c r="G37" s="18" t="n"/>
-      <c r="H37" s="19" t="n"/>
+      <c r="H37" s="18" t="n"/>
+      <c r="I37" s="19" t="n"/>
     </row>
     <row r="38">
-      <c r="D38" s="19" t="n"/>
       <c r="E38" s="19" t="n"/>
-      <c r="F38" s="18" t="n"/>
+      <c r="F38" s="19" t="n"/>
       <c r="G38" s="18" t="n"/>
-      <c r="H38" s="19" t="n"/>
+      <c r="H38" s="18" t="n"/>
+      <c r="I38" s="19" t="n"/>
     </row>
     <row r="39">
-      <c r="D39" s="19" t="n"/>
       <c r="E39" s="19" t="n"/>
-      <c r="F39" s="18" t="n"/>
+      <c r="F39" s="19" t="n"/>
       <c r="G39" s="18" t="n"/>
-      <c r="H39" s="19" t="n"/>
+      <c r="H39" s="18" t="n"/>
+      <c r="I39" s="19" t="n"/>
     </row>
     <row r="40">
-      <c r="D40" s="19" t="n"/>
       <c r="E40" s="19" t="n"/>
-      <c r="F40" s="18" t="n"/>
+      <c r="F40" s="19" t="n"/>
       <c r="G40" s="18" t="n"/>
-      <c r="H40" s="19" t="n"/>
+      <c r="H40" s="18" t="n"/>
+      <c r="I40" s="19" t="n"/>
     </row>
     <row r="41">
-      <c r="D41" s="19" t="n"/>
       <c r="E41" s="19" t="n"/>
-      <c r="F41" s="18" t="n"/>
+      <c r="F41" s="19" t="n"/>
       <c r="G41" s="18" t="n"/>
-      <c r="H41" s="19" t="n"/>
+      <c r="H41" s="18" t="n"/>
+      <c r="I41" s="19" t="n"/>
     </row>
     <row r="42">
-      <c r="D42" s="19" t="n"/>
       <c r="E42" s="19" t="n"/>
-      <c r="F42" s="18" t="n"/>
+      <c r="F42" s="19" t="n"/>
       <c r="G42" s="18" t="n"/>
-      <c r="H42" s="19" t="n"/>
+      <c r="H42" s="18" t="n"/>
+      <c r="I42" s="19" t="n"/>
     </row>
     <row r="43">
-      <c r="D43" s="19" t="n"/>
       <c r="E43" s="19" t="n"/>
-      <c r="F43" s="18" t="n"/>
+      <c r="F43" s="19" t="n"/>
       <c r="G43" s="18" t="n"/>
-      <c r="H43" s="19" t="n"/>
+      <c r="H43" s="18" t="n"/>
+      <c r="I43" s="19" t="n"/>
     </row>
     <row r="44">
-      <c r="D44" s="19" t="n"/>
       <c r="E44" s="19" t="n"/>
-      <c r="F44" s="18" t="n"/>
+      <c r="F44" s="19" t="n"/>
       <c r="G44" s="18" t="n"/>
-      <c r="H44" s="19" t="n"/>
+      <c r="H44" s="18" t="n"/>
+      <c r="I44" s="19" t="n"/>
     </row>
     <row r="45">
-      <c r="D45" s="19" t="n"/>
       <c r="E45" s="19" t="n"/>
-      <c r="F45" s="18" t="n"/>
+      <c r="F45" s="19" t="n"/>
       <c r="G45" s="18" t="n"/>
-      <c r="H45" s="19" t="n"/>
+      <c r="H45" s="18" t="n"/>
+      <c r="I45" s="19" t="n"/>
     </row>
     <row r="46">
-      <c r="D46" s="19" t="n"/>
       <c r="E46" s="19" t="n"/>
-      <c r="F46" s="18" t="n"/>
+      <c r="F46" s="19" t="n"/>
       <c r="G46" s="18" t="n"/>
-      <c r="H46" s="19" t="n"/>
+      <c r="H46" s="18" t="n"/>
+      <c r="I46" s="19" t="n"/>
     </row>
     <row r="47">
-      <c r="D47" s="19" t="n"/>
       <c r="E47" s="19" t="n"/>
-      <c r="F47" s="18" t="n"/>
+      <c r="F47" s="19" t="n"/>
       <c r="G47" s="18" t="n"/>
-      <c r="H47" s="19" t="n"/>
+      <c r="H47" s="18" t="n"/>
+      <c r="I47" s="19" t="n"/>
     </row>
     <row r="48">
-      <c r="D48" s="19" t="n"/>
       <c r="E48" s="19" t="n"/>
-      <c r="F48" s="18" t="n"/>
+      <c r="F48" s="19" t="n"/>
       <c r="G48" s="18" t="n"/>
-      <c r="H48" s="19" t="n"/>
+      <c r="H48" s="18" t="n"/>
+      <c r="I48" s="19" t="n"/>
     </row>
     <row r="49">
-      <c r="D49" s="19" t="n"/>
       <c r="E49" s="19" t="n"/>
-      <c r="F49" s="18" t="n"/>
+      <c r="F49" s="19" t="n"/>
       <c r="G49" s="18" t="n"/>
-      <c r="H49" s="19" t="n"/>
+      <c r="H49" s="18" t="n"/>
+      <c r="I49" s="19" t="n"/>
     </row>
     <row r="50">
-      <c r="D50" s="19" t="n"/>
       <c r="E50" s="19" t="n"/>
-      <c r="F50" s="18" t="n"/>
+      <c r="F50" s="19" t="n"/>
       <c r="G50" s="18" t="n"/>
-      <c r="H50" s="19" t="n"/>
+      <c r="H50" s="18" t="n"/>
+      <c r="I50" s="19" t="n"/>
     </row>
     <row r="51">
-      <c r="D51" s="19" t="n"/>
       <c r="E51" s="19" t="n"/>
-      <c r="F51" s="18" t="n"/>
+      <c r="F51" s="19" t="n"/>
       <c r="G51" s="18" t="n"/>
-      <c r="H51" s="19" t="n"/>
+      <c r="H51" s="18" t="n"/>
+      <c r="I51" s="19" t="n"/>
     </row>
     <row r="52">
-      <c r="D52" s="19" t="n"/>
       <c r="E52" s="19" t="n"/>
-      <c r="F52" s="18" t="n"/>
+      <c r="F52" s="19" t="n"/>
       <c r="G52" s="18" t="n"/>
-      <c r="H52" s="19" t="n"/>
+      <c r="H52" s="18" t="n"/>
+      <c r="I52" s="19" t="n"/>
     </row>
     <row r="53">
-      <c r="D53" s="19" t="n"/>
       <c r="E53" s="19" t="n"/>
-      <c r="F53" s="18" t="n"/>
+      <c r="F53" s="19" t="n"/>
       <c r="G53" s="18" t="n"/>
-      <c r="H53" s="19" t="n"/>
+      <c r="H53" s="18" t="n"/>
+      <c r="I53" s="19" t="n"/>
     </row>
     <row r="54">
-      <c r="D54" s="19" t="n"/>
       <c r="E54" s="19" t="n"/>
-      <c r="F54" s="18" t="n"/>
+      <c r="F54" s="19" t="n"/>
       <c r="G54" s="18" t="n"/>
-      <c r="H54" s="19" t="n"/>
+      <c r="H54" s="18" t="n"/>
+      <c r="I54" s="19" t="n"/>
     </row>
     <row r="55">
-      <c r="D55" s="19" t="n"/>
       <c r="E55" s="19" t="n"/>
-      <c r="F55" s="18" t="n"/>
+      <c r="F55" s="19" t="n"/>
       <c r="G55" s="18" t="n"/>
-      <c r="H55" s="19" t="n"/>
+      <c r="H55" s="18" t="n"/>
+      <c r="I55" s="19" t="n"/>
     </row>
     <row r="56">
-      <c r="D56" s="19" t="n"/>
       <c r="E56" s="19" t="n"/>
-      <c r="F56" s="18" t="n"/>
+      <c r="F56" s="19" t="n"/>
       <c r="G56" s="18" t="n"/>
-      <c r="H56" s="19" t="n"/>
+      <c r="H56" s="18" t="n"/>
+      <c r="I56" s="19" t="n"/>
     </row>
     <row r="57">
-      <c r="D57" s="19" t="n"/>
       <c r="E57" s="19" t="n"/>
-      <c r="F57" s="18" t="n"/>
+      <c r="F57" s="19" t="n"/>
       <c r="G57" s="18" t="n"/>
-      <c r="H57" s="19" t="n"/>
+      <c r="H57" s="18" t="n"/>
+      <c r="I57" s="19" t="n"/>
     </row>
     <row r="58">
-      <c r="D58" s="19" t="n"/>
       <c r="E58" s="19" t="n"/>
-      <c r="F58" s="18" t="n"/>
+      <c r="F58" s="19" t="n"/>
       <c r="G58" s="18" t="n"/>
-      <c r="H58" s="19" t="n"/>
+      <c r="H58" s="18" t="n"/>
+      <c r="I58" s="19" t="n"/>
     </row>
     <row r="59">
-      <c r="D59" s="19" t="n"/>
       <c r="E59" s="19" t="n"/>
-      <c r="F59" s="18" t="n"/>
+      <c r="F59" s="19" t="n"/>
       <c r="G59" s="18" t="n"/>
-      <c r="H59" s="19" t="n"/>
+      <c r="H59" s="18" t="n"/>
+      <c r="I59" s="19" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H4"/>
+  <autoFilter ref="A3:J59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>